<commit_message>
fix(review): ship stable uuids in the sample manual
Review finding 2: without a uuid column every fresh copy got new ids, so a re-sync deleted and re-embedded all 60 rows. The uuids are uuid5 of each question under a fixed namespace.
</commit_message>
<xml_diff>
--- a/examples/carbonm_sample_manual.xlsx
+++ b/examples/carbonm_sample_manual.xlsx
@@ -413,11 +413,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -431,6 +432,11 @@
           <t>answer</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -443,6 +449,11 @@
           <t>答：在登入畫面點選「忘記密碼？」，輸入帳號綁定的公司信箱後按「寄送重設信」。系統會在 5 分鐘內寄出重設連結，連結 30 分鐘內有效，點開後即可設定新密碼。</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>9ffd7433-66ec-560a-b220-799e6f41c2ca</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -455,6 +466,11 @@
           <t>答：密碼長度需為 10 到 20 個字元，至少包含英文字母、數字與符號各一種，且不得與前 3 次使用過的密碼相同。</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>00254f79-9e30-5426-9429-bedde61d92d8</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -467,6 +483,11 @@
           <t>答：開啟公司專屬的 CarbonM 網址，輸入帳號（公司信箱）與密碼後按「登入」。若公司啟用單一登入，請改點「使用公司帳號登入」。</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>29f97434-1b75-57f7-ba54-8cf647f106ec</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -479,6 +500,11 @@
           <t>答：連續輸入錯誤密碼 5 次，帳號會被鎖定 15 分鐘。鎖定期間可以使用「忘記密碼？」重設密碼，或請系統管理者手動解鎖。</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>03ff9102-19a1-51c7-8960-b7fd8f029138</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -491,6 +517,11 @@
           <t>答：點選右上角頭像，選擇「個人設定」，即可修改顯示名稱、聯絡電話與通知偏好。帳號信箱由系統管理者設定，使用者無法自行修改。</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0f6af7a0-421a-5a3e-9256-02abef18fff7</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -503,6 +534,11 @@
           <t>答：點選右上角頭像，選擇「登出」。閒置超過 60 分鐘，系統也會自動登出。</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>fa5efdd7-3848-58b6-967a-1c38eb8f30a4</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -515,6 +551,11 @@
           <t>答：CarbonM 有三種角色：系統管理者可管理帳號與組織設定；廠區負責人可管理所屬廠區的排放源並審核數據；填報人員只能填寫與修改自己負責的數據條目。</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>a1e33d67-db7c-5a4b-b627-87122cfc5730</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -527,6 +568,11 @@
           <t>答：系統管理者進入「組織設定」&gt;「帳號管理」，點選「新增使用者」，填寫姓名、公司信箱、角色與所屬廠區後儲存。系統會寄送啟用信給新使用者。</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1ee541c3-5a5d-5e95-b5de-142c8fe53de4</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -539,6 +585,11 @@
           <t>答：啟用信 7 天內有效。過期後請系統管理者在「帳號管理」找到該使用者，點選「重新寄送啟用信」。</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>e49e7add-ed60-554a-896e-a0b5ba8264dc</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -551,6 +602,11 @@
           <t>答：進入「個人設定」&gt;「安全性」，點選「啟用兩步驟驗證」，用驗證器 App 掃描 QR Code 並輸入 6 位數驗證碼即可完成。</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>4e7e0918-095c-5e5e-bcac-6ff78d757dbd</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -563,6 +619,11 @@
           <t>答：系統管理者在「帳號管理」找到該使用者，點選「停用」。停用後帳號無法登入，但其填報過的數據與審核紀錄會保留。</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>f18094aa-d223-5d15-9053-7ac06e0d1722</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -575,6 +636,11 @@
           <t>答：可以。系統管理者在編輯使用者時可勾選多個所屬廠區，使用者登入後可從畫面上方的廠區選單切換。</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2fbc5b52-71a3-5a51-b8fa-81f7c4015ef9</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -587,6 +653,11 @@
           <t>答：盤查邊界是指這次溫室氣體盤查要涵蓋的範圍，包含組織邊界（哪些公司或廠區納入）與營運邊界（納入哪些排放類別）。</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>fb071fae-6215-5324-93eb-30314e8a5dfc</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -599,6 +670,11 @@
           <t>答：CarbonM 支援營運控制法、財務控制法與股權比例法。設定位置在「組織設定」&gt;「盤查邊界」，選定方法後，系統會依各廠區的控制或持股比例計算納入量。</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>08b14e88-7e51-5918-b78c-344adef1c9b3</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -611,6 +687,11 @@
           <t>答：系統管理者進入「組織設定」&gt;「廠區管理」，點選「新增廠區」，填寫廠區名稱、地址、產業類別與啟用年度後儲存。</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>71ee2949-f868-57d7-817b-eba1b486d10d</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -623,6 +704,11 @@
           <t>答：在「組織設定」&gt;「盤查邊界」選擇盤查年度後，勾選或取消要納入的廠區並按「套用」。切換只影響該年度，不會改變其他年度已完成的盤查。</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>55c85fb8-df67-52db-8627-9613d703e02b</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -635,6 +721,11 @@
           <t>答：在「廠區管理」使用「合併廠區」或「分割廠區」功能，並指定生效日期。生效日前的數據保留在原廠區，生效日後的數據歸入新的廠區。</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>22bac8a0-d822-5fc8-982a-8e47c30f62c5</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -647,6 +738,11 @@
           <t>答：基準年是用來比較減量成效的參考年度。可在「盤查邊界」設定，設定後若組織邊界有重大變動，系統會提示是否需要重新計算基準年排放量。</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>5de71dc4-3ee3-5519-ae58-0c03c17ded83</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -659,6 +755,11 @@
           <t>答：在「組織設定」&gt;「盤查年度」點選「新增年度」，選擇起訖日期（預設為 1 月 1 日至 12 月 31 日），並指定要沿用哪一個年度的邊界設定。</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>8988420e-e34d-5a12-a8ad-df58ffde4035</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -671,6 +772,11 @@
           <t>答：營運邊界分為範疇一（直接排放）、範疇二（外購能源的間接排放）與範疇三（其他間接排放）。範疇一與範疇二為必填，範疇三可依需求勾選要納入的類別。</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>4918f224-d416-5b01-b497-c079a96a0a54</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -683,6 +789,11 @@
           <t>答：可以。在「排放源管理」將該排放源標記為「排除」並填寫排除理由。排除的排放量合計超過總排放量 5% 時，系統會顯示警示。</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>c5036131-9924-51a7-86f0-e87e8b2271bf</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -695,6 +806,11 @@
           <t>答：依組織邊界方法決定。採營運控制法時，若公司對該辦公室具有營運控制權，就應將其用電與冷媒等排放納入盤查。</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>8b35fcf8-f6ce-5784-99c8-f3abbcc5fac2</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -707,6 +823,11 @@
           <t>答：新增盤查年度時，在「沿用設定」選擇去年的年度，系統會複製廠區清單、邊界方法與排放源設定，數據條目則不會複製。</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ead8ad49-9964-5828-a5f5-06c9ce7ef54d</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -719,6 +840,11 @@
           <t>答：系統管理者可以檢視全部廠區；廠區負責人與填報人員只能看到自己所屬的廠區。</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>24cd7fce-f1b2-56e1-a43b-c0c526579515</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -731,6 +857,11 @@
           <t>答：固定式燃料源排放是指在固定設備中燃燒燃料所產生的直接排放，例如鍋爐、發電機與加熱爐燃燒天然氣、柴油或燃料油，屬於範疇一。</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>3ccbfd72-ffb7-5226-a9ec-6cff4f75897f</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -743,6 +874,11 @@
           <t>答：移動源排放是指公司擁有或控制的交通工具燃燒燃料所產生的排放，例如公務車、堆高機與貨車使用汽油或柴油，屬於範疇一。</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>d4645c9c-a95e-55a8-8b67-b3daf6a9d1c0</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -755,6 +891,11 @@
           <t>答：外購電力排放是指公司向電力公司購買並使用的電力，在發電端所產生的間接排放，屬於範疇二。計算方式為用電度數乘以電力排放係數。</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>4d4dfb84-86c8-5bba-a909-ad29b873634f</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -767,6 +908,11 @@
           <t>答：冷媒逸散屬於範疇一。CarbonM 提供兩種方式：有補充紀錄時使用「填充量法」，以年度補充量乘以該冷媒的 GWP；沒有紀錄時使用「設備逸散率法」，以設備原始填充量乘以預設逸散率再乘以 GWP。</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2549a037-9754-55ec-ba11-bcf746fa7a71</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -779,6 +925,11 @@
           <t>答：排放係數是將活動數據換算為溫室氣體排放量的比率，例如每公升柴油或每度電會產生多少公斤二氧化碳當量。</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>6498d787-680a-5629-8983-bd6e02829c93</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -791,6 +942,11 @@
           <t>答：CarbonM 內建「係數庫」，收錄官方公告的燃料、電力與冷媒係數，並標示來源與適用年度。系統預設使用與盤查年度相符的最新版本。</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>3fdfe0a0-ef7e-5980-9df8-c6f5d526ccf2</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -803,6 +959,11 @@
           <t>答：可以。在「係數庫」點選「新增自訂係數」，填寫係數值、單位與來源文件後送出，經系統管理者核准即可在排放源中選用。</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>edc5d170-c404-5b24-a843-ab3ef280afcb</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -815,6 +976,11 @@
           <t>答：GWP（全球暖化潛勢）表示某種溫室氣體在特定期間內造成的暖化效果相當於多少單位的二氧化碳。CarbonM 預設採用 100 年期的 GWP 值。</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>c825bec0-fab0-54b0-9bd0-75fa9062885a</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -827,6 +993,11 @@
           <t>答：進入「排放源管理」，選擇廠區後點選「新增排放源」，依序選擇範疇、排放類別、燃料或物料種類與排放係數，填寫設備名稱後儲存。</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>c24d9a90-2889-540a-a979-8f47ccf53ff3</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -839,6 +1010,11 @@
           <t>答：活動數據是造成排放的活動量，例如燃料使用量、用電度數或冷媒補充量。活動數據乘以排放係數就能得到排放量。</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>e3b4b001-61a2-51b4-b77d-cbca385f68c8</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -851,6 +1027,11 @@
           <t>答：化糞池產生的甲烷屬於範疇一的逸散排放。若廠區使用化糞池處理生活污水，應以員工人數與工作天數估算並納入盤查。</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>a6764b7d-b6a8-5710-8002-05a39b1628ac</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -863,6 +1044,11 @@
           <t>答：常見的範疇三類別包括上游運輸、員工通勤、商務差旅、購買的商品與服務，以及廢棄物處理。CarbonM 可在營運邊界中逐項勾選要納入的類別。</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>7b662ee3-0d5f-5df7-9a7a-91aa05a8a4d6</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -875,6 +1061,11 @@
           <t>答：進入「數據填報」，選擇盤查年度、廠區與排放源後點選「新增數據條目」，填寫期間、活動數據與單位，並上傳佐證文件（例如帳單或發票）後送出。</t>
         </is>
       </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>8ba09eef-df50-5fc6-8885-49f9119a1618</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -887,6 +1078,11 @@
           <t>答：可以。在「數據填報」點選「批次匯入」，下載範本並依欄位填寫後上傳 XLSX 或 CSV。系統會先檢查格式，有錯誤的列會標示原因，修正後再重新上傳。</t>
         </is>
       </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>00603901-e35c-567a-9a48-31a0245c1389</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -899,6 +1095,11 @@
           <t>答：廠區負責人進入「審核中心」，在待審核清單中點開數據條目，檢查活動數據與佐證文件後選擇「核准」或「退回」。退回時必須填寫原因。</t>
         </is>
       </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2ecf8141-e2cf-5ef8-a32a-218eedcbb08b</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -911,6 +1112,11 @@
           <t>答：填報人員會收到通知，可以在「數據填報」的「已退回」分頁查看退回原因，修正內容或補上佐證文件後重新送出。</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ea176a3d-d131-5553-8589-3487e92faa3e</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -923,6 +1129,11 @@
           <t>答：已核准的數據條目會被鎖定。如需修改，請廠區負責人在「審核中心」點選「解除核准」並填寫理由，數據會回到填報人員手上修改。</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>20fab90f-84ee-55d6-a803-9b51e352a3fb</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -935,6 +1146,11 @@
           <t>答：佐證文件支援 PDF、JPG、PNG、XLSX 與 CSV，單一檔案上限 20 MB，每筆數據條目最多可上傳 5 個檔案。</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>939113ef-f38c-5dbc-9e8c-4cfb013301bd</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -947,6 +1163,11 @@
           <t>答：會。數據送出時，系統會將其與同一排放源的前 12 個月平均比較，差異超過 30% 時標示為「異常」，提醒審核者特別確認。</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>fb24e8f3-efec-5c0a-9b4f-885a85bde902</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -959,6 +1180,11 @@
           <t>答：數據品質等級用來表示活動數據的可信程度，分為「實測」「帳單」「估算」三級。審核者可依等級判斷是否需要補充佐證。</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>f7573e31-c16e-585d-b884-6c23e3662a7d</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -971,6 +1197,11 @@
           <t>答：在數據條目的詳細頁面點選「歷程」分頁，可以看到每次修改的時間、修改者、修改前後的數值與審核紀錄。</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>eab29522-da6f-53cb-87c1-2c24067b3402</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -983,6 +1214,11 @@
           <t>答：系統管理者在「盤查年度」設定中填寫「填報截止日」。截止日前 7 天，系統會提醒尚未完成填報的人員。</t>
         </is>
       </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>26703a08-f783-5376-868a-30fc9bdc03bb</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -995,6 +1231,11 @@
           <t>答：可以。廠區負責人在「個人設定」&gt;「代理設定」選擇代理人與代理期間，期間內代理人可以審核該廠區的數據條目。</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2cdd9e30-d395-5136-a39e-ea707d8d33e5</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1007,6 +1248,11 @@
           <t>答：在「審核中心」的「進度總覽」可以看到各廠區、各排放源的填報與審核進度。全部顯示「已核准」後，才能產生正式的盤查報告。</t>
         </is>
       </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ca3a8788-4367-59bd-8688-2b97804d468f</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1019,6 +1265,11 @@
           <t>答：CarbonM 可匯出溫室氣體盤查清冊（XLSX）與盤查報告書（DOCX 與 PDF）。清冊列出每個排放源的活動數據、係數與排放量，報告書則包含邊界說明、方法學與排放量彙總。</t>
         </is>
       </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>fd39270d-688d-5799-bc5b-f9fc46d6f6d7</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1031,6 +1282,11 @@
           <t>答：進入「報表中心」，選擇盤查年度後點選「產生報告書」。系統會檢查數據是否已全部核准，通過後約 1 至 3 分鐘即可下載。</t>
         </is>
       </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>b51ff1ed-8077-5e96-9e69-46424fc23903</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1043,6 +1299,11 @@
           <t>答：報告書中的排放數據由系統計算產生，無法直接修改；公司簡介、減量措施等文字段落可以在「報表中心」的「報告書設定」編輯後重新產生。</t>
         </is>
       </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>17b8f656-aecb-56c5-bd18-9976be168d0f</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1055,6 +1316,11 @@
           <t>答：儀表板顯示年度總排放量、各範疇占比、各廠區排放排名與逐月趨勢，並可與基準年比較減量進度。</t>
         </is>
       </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>dd05a4fc-71bb-56ba-a016-5538eab08b65</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1067,6 +1333,11 @@
           <t>答：在「儀表板」點選「年度比較」，勾選要比較的年度，系統會以長條圖呈現各範疇與各廠區的差異。</t>
         </is>
       </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>09f6e7ce-c7b9-513a-bb63-09c3e56be271</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1079,6 +1350,11 @@
           <t>答：可以。在「報表中心」點選「匯出原始數據」，選擇年度與廠區後下載 CSV，內容包含所有已核准的數據條目。</t>
         </is>
       </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>ff1c977c-c38f-539e-8d7f-154896f2663f</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1091,6 +1367,11 @@
           <t>答：排放強度是排放量除以營運指標的比值，例如每百萬元營收或每噸產品的排放量。可在「報表中心」&gt;「強度指標」設定分母後自動計算。</t>
         </is>
       </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>826b8837-ea24-5ca4-94fa-66cb19eb7da9</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1103,6 +1384,11 @@
           <t>答：報告書的排放量統一以公噸二氧化碳當量（tCO2e）呈現，小數點以下保留 3 位。</t>
         </is>
       </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>16540266-2a8f-5bec-b520-23f794dc3a86</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1115,6 +1401,11 @@
           <t>答：可以。在「報表中心」&gt;「排程寄送」設定報表類型、寄送頻率（每月或每季）與收件人，系統會依排程寄出 PDF 摘要。</t>
         </is>
       </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>15bda7ee-a652-5aca-a37f-40bc88d71847</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1127,6 +1418,11 @@
           <t>答：在「報表中心」點選「查證資料包」，系統會將清冊、報告書、佐證文件與數據修改紀錄打包成一個壓縮檔，可提供給查證機構。</t>
         </is>
       </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>4a873f79-ac92-5b1a-8c41-234ce379ed65</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1139,6 +1435,11 @@
           <t>答：最常見的原因是仍有未核准的數據條目。請先到「審核中心」的「進度總覽」確認；若全部已核准仍失敗，請記下畫面上的錯誤代碼並聯絡系統管理者。</t>
         </is>
       </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>8f19ab79-bc0f-5269-965e-806e5b01ac6a</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1149,6 +1450,11 @@
       <c r="B61" t="inlineStr">
         <is>
           <t>答：儀表板即時包含尚未核准的數據，清冊只計算已核准的數據條目。兩者不同通常代表仍有待審核或被退回的數據。</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>0ad7a904-17f5-58f9-9474-4348009f781d</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: remove remaining text from the third-party manual
Replace two test fixtures and an old proposal example that quoted the previous manual, and reword three sample-manual questions that matched it verbatim.
</commit_message>
<xml_diff>
--- a/examples/carbonm_sample_manual.xlsx
+++ b/examples/carbonm_sample_manual.xlsx
@@ -696,7 +696,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>16. 問：如何在多廠區管理中切換邊界？</t>
+          <t>16. 問：多廠區要怎麼切換盤查邊界？</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>55c85fb8-df67-52db-8627-9613d703e02b</t>
+          <t>f66e7b40-bb63-5175-9ea6-e18e1d07667e</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>27. 問：「外購電力」排放代表什麼？</t>
+          <t>27. 問：外購電力的排放代表什麼？</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>4d4dfb84-86c8-5bba-a909-ad29b873634f</t>
+          <t>73df7549-7314-51a5-a951-ce5a3d3326a7</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>39. 問：我該如何審核數據條目？</t>
+          <t>39. 問：如何審核數據條目？</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2ecf8141-e2cf-5ef8-a32a-218eedcbb08b</t>
+          <t>fdceb39a-3a54-5545-a7ea-1604ba1adf9a</t>
         </is>
       </c>
     </row>

</xml_diff>